<commit_message>
chore(sync): synchronize live broker fill META and working AVGO state from VPS
</commit_message>
<xml_diff>
--- a/shared/SkonVault_Live_Transaction_Journal.xlsx
+++ b/shared/SkonVault_Live_Transaction_Journal.xlsx
@@ -174,7 +174,7 @@
     <row r="2">
       <c r="A2" t="inlineStr" s="2">
         <is>
-          <t>Executive Live Telemetry: 72h Weekend Theta Compounding &amp; Rollover Radar — As of 2026-09-29 17:41 ICT</t>
+          <t>Executive Live Telemetry: 72h Weekend Theta Compounding &amp; Rollover Radar — As of 2026-09-29 21:21 ICT</t>
         </is>
       </c>
     </row>
@@ -212,19 +212,19 @@
     </row>
     <row r="5">
       <c r="A5" s="6">
-        <v>32632.58</v>
+        <v>32729.7</v>
       </c>
       <c r="C5" s="6">
         <v>0.0</v>
       </c>
       <c r="E5" s="7">
-        <v>612.0</v>
+        <v>710.0</v>
       </c>
       <c r="G5" s="7">
-        <v>306.0</v>
+        <v>355.0</v>
       </c>
       <c r="I5" s="6">
-        <v>3700.0</v>
+        <v>4200.0</v>
       </c>
       <c r="K5" t="inlineStr" s="10">
         <is>
@@ -334,11 +334,11 @@
         <v>6</v>
       </c>
       <c r="F8" s="6">
-        <v>228.86</v>
+        <v>229.93</v>
       </c>
       <c r="G8" t="inlineStr" s="7">
         <is>
-          <t>+$8.86 (+3.9%) OTM Buffer 🟢</t>
+          <t>+$9.93 (+4.3%) OTM Buffer 🟢</t>
         </is>
       </c>
       <c r="H8" s="6">
@@ -397,11 +397,11 @@
         <v>1</v>
       </c>
       <c r="F9" s="6">
-        <v>62.1</v>
+        <v>61.67</v>
       </c>
       <c r="G9" t="inlineStr" s="7">
         <is>
-          <t>+$2.10 (+3.4%) OTM Buffer 🟢</t>
+          <t>+$1.67 (+2.7%) OTM Buffer 🟢</t>
         </is>
       </c>
       <c r="H9" s="6">
@@ -438,12 +438,12 @@
     <row r="10">
       <c r="A10" t="inlineStr" s="0">
         <is>
-          <t>1. AI Chips &amp; Hardware</t>
+          <t>8. Mega-Cap Cloud &amp; Software Platform</t>
         </is>
       </c>
       <c r="B10" t="inlineStr" s="10">
         <is>
-          <t>TSM</t>
+          <t>META</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="0">
@@ -453,83 +453,146 @@
       </c>
       <c r="D10" t="inlineStr" s="10">
         <is>
-          <t>$425.00P / $420.00P</t>
+          <t>$685.00P / $680.00P</t>
         </is>
       </c>
       <c r="E10" s="0">
         <v>1</v>
       </c>
       <c r="F10" s="6">
-        <v>452.88</v>
+        <v>721.195</v>
       </c>
       <c r="G10" t="inlineStr" s="7">
         <is>
-          <t>+$27.88 (+6.2%) OTM Buffer 🟢</t>
+          <t>+$36.20 (+5.0%) OTM Buffer 🟢</t>
         </is>
       </c>
       <c r="H10" s="6">
-        <v>897.0</v>
+        <v>555.0</v>
       </c>
       <c r="I10" s="6">
-        <v>747.0</v>
+        <v>457.0</v>
       </c>
       <c r="J10" s="7">
-        <v>150.0</v>
+        <v>98.0</v>
       </c>
       <c r="K10" s="7">
-        <v>75.0</v>
+        <v>49.0</v>
       </c>
       <c r="L10" s="6">
         <v>500.0</v>
       </c>
       <c r="M10" t="inlineStr" s="0">
         <is>
+          <t>Oct 06, 2026 (T-3 DTE)</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr" s="0">
+        <is>
+          <t>Oct 09, 2026</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr" s="7">
+        <is>
+          <t>100% SAFE (Theta Burning on Schedule) 🟢</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr" s="0">
+        <is>
+          <t>1. AI Chips &amp; Hardware</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr" s="10">
+        <is>
+          <t>TSM</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr" s="0">
+        <is>
+          <t>Tradier Live (#6YB80974)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr" s="10">
+        <is>
+          <t>$425.00P / $420.00P</t>
+        </is>
+      </c>
+      <c r="E11" s="0">
+        <v>1</v>
+      </c>
+      <c r="F11" s="6">
+        <v>454.855</v>
+      </c>
+      <c r="G11" t="inlineStr" s="7">
+        <is>
+          <t>+$29.86 (+6.6%) OTM Buffer 🟢</t>
+        </is>
+      </c>
+      <c r="H11" s="6">
+        <v>897.0</v>
+      </c>
+      <c r="I11" s="6">
+        <v>747.0</v>
+      </c>
+      <c r="J11" s="7">
+        <v>150.0</v>
+      </c>
+      <c r="K11" s="7">
+        <v>75.0</v>
+      </c>
+      <c r="L11" s="6">
+        <v>500.0</v>
+      </c>
+      <c r="M11" t="inlineStr" s="0">
+        <is>
           <t>Oct 27, 2026 (T-3 DTE)</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr" s="0">
+      <c r="N11" t="inlineStr" s="0">
         <is>
           <t>Oct 30, 2026</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr" s="7">
+      <c r="O11" t="inlineStr" s="7">
         <is>
           <t>100% SAFE (Theta Burning on Schedule) 🟢</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr" s="5">
+    <row r="12">
+      <c r="A12" t="inlineStr" s="5">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5">
-        <v>8</v>
-      </c>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5">
-        <v>1991.0</v>
-      </c>
-      <c r="I11" s="5">
-        <v>1379.0</v>
-      </c>
-      <c r="J11" s="5">
-        <v>612.0</v>
-      </c>
-      <c r="K11" s="5">
-        <v>306.0</v>
-      </c>
-      <c r="L11" s="5">
-        <v>3700.0</v>
-      </c>
-      <c r="M11" s="5"/>
-      <c r="N11" s="5"/>
-      <c r="O11" t="inlineStr" s="5">
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5">
+        <v>9</v>
+      </c>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="5">
+        <v>2546.0</v>
+      </c>
+      <c r="I12" s="5">
+        <v>1836.0</v>
+      </c>
+      <c r="J12" s="5">
+        <v>710.0</v>
+      </c>
+      <c r="K12" s="5">
+        <v>355.0</v>
+      </c>
+      <c r="L12" s="5">
+        <v>4200.0</v>
+      </c>
+      <c r="M12" s="5"/>
+      <c r="N12" s="5"/>
+      <c r="O12" t="inlineStr" s="5">
         <is>
           <t>100% DEFINED RISK PROTECTED ✅</t>
         </is>
@@ -1257,6 +1320,116 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr" s="0">
+        <is>
+          <t>TRD-20260929-META-685/680</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr" s="0">
+        <is>
+          <t>Tradier Live (#6YB80974)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr" s="10">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr" s="0">
+        <is>
+          <t>8. Mega-Cap Cloud &amp; Software Platform</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr" s="0">
+        <is>
+          <t>Bull Put Spread (685P/680P)</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr" s="0">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr" s="0">
+        <is>
+          <t>14:16:18</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr" s="0">
+        <is>
+          <t>META261009P00685000</t>
+        </is>
+      </c>
+      <c r="I10" s="6">
+        <v>685.0</v>
+      </c>
+      <c r="J10" t="inlineStr" s="0">
+        <is>
+          <t>META261009P00680000</t>
+        </is>
+      </c>
+      <c r="K10" s="6">
+        <v>680.0</v>
+      </c>
+      <c r="L10" t="inlineStr" s="0">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M10" s="0">
+        <v>1</v>
+      </c>
+      <c r="N10" s="6">
+        <v>0.98</v>
+      </c>
+      <c r="O10" s="6">
+        <v>98.0</v>
+      </c>
+      <c r="P10" s="6">
+        <v>500.0</v>
+      </c>
+      <c r="Q10" t="inlineStr" s="0">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr" s="0">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S10" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="T10" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="U10" s="7">
+        <v>98.0</v>
+      </c>
+      <c r="V10" s="8">
+        <v>0.196</v>
+      </c>
+      <c r="W10" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="X10" t="inlineStr" s="0">
+        <is>
+          <t>Active with broker (live position)</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr" s="10">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr" s="0">
+        <is>
+          <t>148305471</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -1602,6 +1775,56 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr" s="0">
+        <is>
+          <t>TAX-20260929-META-685/680</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr" s="0">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr" s="0">
+        <is>
+          <t>Tradier (Apex Clearing Corp)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr" s="0">
+        <is>
+          <t>6YB80974</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr" s="10">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="F10" s="6">
+        <v>98.0</v>
+      </c>
+      <c r="G10" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="H10" s="7">
+        <v>98.0</v>
+      </c>
+      <c r="I10" s="6">
+        <v>36.5</v>
+      </c>
+      <c r="J10" s="9">
+        <v>3577.0</v>
+      </c>
+      <c r="K10" s="9">
+        <v>3577.0</v>
+      </c>
+      <c r="L10" t="inlineStr" s="0">
+        <is>
+          <t>148305471</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>